<commit_message>
Complete today's RepoMaster work
</commit_message>
<xml_diff>
--- a/templates/Vehicle_Template.xlsx
+++ b/templates/Vehicle_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A322A65-C6E6-4468-A86E-F67853B3AB16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2802892A-B049-41EB-BB75-4D58AFDBF4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Repo Year</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Chassis Number</t>
   </si>
   <si>
-    <t>Color</t>
-  </si>
-  <si>
     <t>Vehicle Make</t>
   </si>
   <si>
@@ -109,9 +106,6 @@
     <t>Agency ID</t>
   </si>
   <si>
-    <t>Ref Letter</t>
-  </si>
-  <si>
     <t>Total Charges</t>
   </si>
   <si>
@@ -140,6 +134,9 @@
   </si>
   <si>
     <t>AgencyID give by Finance</t>
+  </si>
+  <si>
+    <t>Vehicle Color</t>
   </si>
 </sst>
 </file>
@@ -479,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AN1"/>
+  <dimension ref="A1:AM1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" customWidth="1"/>
@@ -489,6 +486,7 @@
     <col min="5" max="5" width="14.85546875" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
     <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="11" width="14.28515625" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
@@ -509,14 +507,13 @@
     <col min="32" max="32" width="21.42578125" customWidth="1"/>
     <col min="33" max="33" width="33.140625" customWidth="1"/>
     <col min="34" max="34" width="29.140625" customWidth="1"/>
-    <col min="35" max="35" width="16.28515625" customWidth="1"/>
-    <col min="36" max="36" width="14.5703125" customWidth="1"/>
-    <col min="37" max="37" width="16.42578125" customWidth="1"/>
-    <col min="38" max="38" width="36" customWidth="1"/>
-    <col min="39" max="39" width="22.140625" customWidth="1"/>
+    <col min="35" max="35" width="14.5703125" customWidth="1"/>
+    <col min="36" max="36" width="16.42578125" customWidth="1"/>
+    <col min="37" max="37" width="36" customWidth="1"/>
+    <col min="38" max="38" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,40 +530,40 @@
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" t="s">
         <v>33</v>
       </c>
-      <c r="I1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K1" t="s">
-        <v>38</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" t="s">
         <v>34</v>
       </c>
-      <c r="M1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" t="s">
         <v>37</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>39</v>
       </c>
       <c r="R1" t="s">
         <v>6</v>
@@ -581,61 +578,58 @@
         <v>5</v>
       </c>
       <c r="V1" t="s">
+        <v>17</v>
+      </c>
+      <c r="W1" t="s">
+        <v>11</v>
+      </c>
+      <c r="X1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z1" t="s">
         <v>18</v>
       </c>
-      <c r="W1" t="s">
-        <v>12</v>
-      </c>
-      <c r="X1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>21</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>22</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>23</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>24</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>25</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>26</v>
       </c>
-      <c r="AH1" t="s">
-        <v>27</v>
-      </c>
       <c r="AI1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AJ1" t="s">
         <v>29</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>30</v>
       </c>
-      <c r="AK1" t="s">
-        <v>31</v>
-      </c>
       <c r="AL1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="AM1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>